<commit_message>
Add taxonomy version filter to articles for improved data selection
</commit_message>
<xml_diff>
--- a/data/meso_samples_4validation.xlsx
+++ b/data/meso_samples_4validation.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:E101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,10 +441,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>validation_link</t>
         </is>
@@ -453,68 +458,75 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>migrants and religion</t>
+          <t>public opinion on migration</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Protecting religious freedom of migrants is a moral duty</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>My Lords, a phrase in Deuteronomy 26:5 has long puzzled scholars. It says:
-“A wandering Aramean was my father.”
-I have no time to co...</t>
-        </is>
+          <t>The public is racist about migration</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20a%20phrase%20in%20Deuteronomy%2026%3A5%20has%20long%20puzzled%20scholars.%20It%20says%3A%0D%0A%0D%0A%E2%80%9CA%20wandering%20Aramean%20was%20my%20father.%E2%80%9D%0D%20%0D%0A%0D%0AI%20have%20no%20time%20to%20co...</t>
+          <t>John Cleese criticised for saying London no longer an English city</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=John%20Cleese%20criticised%20for%20saying%20London%20no%20longer%20an%20English%20city</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>migrants and terrorism</t>
+          <t>climate migration</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Small boat arrivals could be terrorists</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>My Lords, I have Amendment 85D in this group and have added my name to Amendment 85C from the noble Lord, Lord Alton, and the amendments fro...</t>
-        </is>
+          <t>Climate change is exaggerated to justify migration</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20have%20Amendment%2085D%20in%20this%20group%20and%20have%20added%20my%20name%20to%20Amendment%2085C%20from%20the%20noble%20Lord%2C%20Lord%20Alton%2C%20and%20the%20amendments%20fro...</t>
+          <t>Poor countries exploit climate panic to press us for easy cash</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Poor%20countries%20exploit%20climate%20panic%20to%20press%20us%20for%20easy%20cash</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migrants and terrorism</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Foreign nationals sentenced to 12 months or more in prison are subject to automatic deportation</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Foreign prisoners in Scottish jails rise amid calls for deportation</t>
-        </is>
+          <t>Attackers in terror attacks are often the children of migrants</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Foreign%20prisoners%20in%20Scottish%20jails%20rise%20amid%20calls%20for%20deportation</t>
+          <t>Shamima Begum's journey from east London schoolgirl to jihadi bride</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Shamima%20Begum%27s%20journey%20from%20east%20London%20schoolgirl%20to%20jihadi%20bride</t>
         </is>
       </c>
     </row>
@@ -526,1317 +538,1497 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Protecting migrants’ human rights benefits the whole society</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>My Lords, it is a privilege to add my voice to this debate. I echo much of what has already been said, including by my friends the most reve...</t>
-        </is>
+          <t>Human rights claims by migrants are often exaggerated</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20it%20is%20a%20privilege%20to%20add%20my%20voice%20to%20this%20debate.%20I%20echo%20much%20of%20what%20has%20already%20been%20said%2C%20including%20by%20my%20friends%20the%20most%20reve...</t>
+          <t>Minister says some human rights claims by migrants 'don't stand up'</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Minister%20says%20some%20human%20rights%20claims%20by%20migrants%20%27don%27t%20stand%20up%27</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>migrants and veterans</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Migrants who serve in the armed forces deserve citizenship</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>My Lords, I am pleased to confirm that the Ministry of Defence has revised its national security vetting policy for all interpreters who dep...</t>
-        </is>
+          <t>Age assessments are unreliable and harm genuine child refugees</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20am%20pleased%20to%20confirm%20that%20the%20Ministry%20of%20Defence%20has%20revised%20its%20national%20security%20vetting%20policy%20for%20all%20interpreters%20who%20dep...</t>
+          <t>&lt;blockquote&gt;&lt;q&gt;1 Before Clause 3, insert the following new clause:&lt;/q&gt;&lt;/blockquote&gt; &lt;blockquote&gt;&lt;q&gt;&lt;em&gt;Young unaccompanied asylum seekers&lt;/e...</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=%3Cblockquote%3E%3Cq%3E1%20Before%20Clause%203%2C%20insert%20the%20following%20new%20clause%3A%3C%2Fq%3E%3C%2Fblockquote%3E%20%3Cblockquote%3E%3Cq%3E%3Cem%3EYoung%20unaccompanied%20asylum%20seekers%3C%2Fe...</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and mental health</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Migrants resist economic integration</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Unless the Federal Government fully funds the resettlement of these refugees . the cost will be passed on to State and local government . Th...</t>
-        </is>
+          <t>Asylum seekers and refugees are especially at risk of developing mental health issues</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Unless%20the%20Federal%20Government%20fully%20funds%20the%20resettlement%20of%20these%20refugees%20.%20the%20cost%20will%20be%20passed%20on%20to%20State%20and%20local%20government%20.%20Th...</t>
+          <t>I would like to start by thanking all those who work with and help asylum seekers and refugees in Newport. They include The Sanctuary projec...</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20would%20like%20to%20start%20by%20thanking%20all%20those%20who%20work%20with%20and%20help%20asylum%20seekers%20and%20refugees%20in%20Newport.%20They%20include%20The%20Sanctuary%20projec...</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>migrants and elections</t>
+          <t>migrants, economy, and labour market</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Migrants influence elections to favour pro-migration parties</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Labour’s plot to diminish democracy</t>
-        </is>
+          <t>Restrictive migration policies increase poverty in host countries</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Labour%E2%80%99s%20plot%20to%20diminish%20democracy</t>
+          <t>Work/Life - international employment news update</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Work%2FLife%20-%20international%20employment%20news%20update</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>small boats and Channel crossings</t>
+          <t>accountability on migration policies</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Rescue operations in the Channel incentivise more crossings</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>My Lords, I speak as a member of the Home Affairs Committee and as a former member of the External Affairs Committee. Migration is a huge gl...</t>
-        </is>
+          <t>There are trade-offs involved in migration policy making</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20speak%20as%20a%20member%20of%20the%20Home%20Affairs%20Committee%20and%20as%20a%20former%20member%20of%20the%20External%20Affairs%20Committee.%20Migration%20is%20a%20huge%20gl...</t>
+          <t>Rwandan President offers to pay back UK money if migrant deal falls through.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rwandan%20President%20offers%20to%20pay%20back%20UK%20money%20if%20migrant%20deal%20falls%20through.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>migrants and crimes</t>
+          <t>border control and sovereignty</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Migrants are involved in child abuse scandals</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Rochdale paedophiles could finally be kicked out of UK after losing court appeal</t>
-        </is>
+          <t>Border control is used to manage migration flows</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rochdale%20paedophiles%20could%20finally%20be%20kicked%20out%20of%20UK%20after%20losing%20court%20appeal</t>
+          <t>I am sure that the noble Baroness has read the Draft Instructions. May I ask her, with all the respect in the world, to read them again? Bec...</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20sure%20that%20the%20noble%20Baroness%20has%20read%20the%20Draft%20Instructions.%20May%20I%20ask%20her%2C%20with%20all%20the%20respect%20in%20the%20world%2C%20to%20read%20them%20again%3F%20Bec...</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>public opinion on migration</t>
+          <t>migrants and elections</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Public opinion supports restricting migration</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Brexiteers and Remainers BOTH wrong about post-Brexit migration - Andrew Neil</t>
-        </is>
+          <t>Commonwealth migrants should not be allowed to vote in UK elections</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Brexiteers%20and%20Remainers%20BOTH%20wrong%20about%20post-Brexit%20migration%20-%20Andrew%20Neil</t>
+          <t>Commonwealth citizens should not be allowed to vote</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Commonwealth%20citizens%20should%20not%20be%20allowed%20to%20vote</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>border control and sovereignty</t>
+          <t>migrants and healthcare system</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Countries have the sovereign right to control their borders</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>I am grateful to the noble Lord for raising those issues. Clause 35 gives the Secretary of State the power to detain a foreign criminal at t...</t>
-        </is>
+          <t>Healthcare access for migrants is a privilege, not a right</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20grateful%20to%20the%20noble%20Lord%20for%20raising%20those%20issues.%20Clause%2035%20gives%20the%20Secretary%20of%20State%20the%20power%20to%20detain%20a%20foreign%20criminal%20at%20t...</t>
+          <t>My hon. Friend, who I am sure will be able to develop his argument further—[HON. MEMBERS:"Oh".] I was referring to the fact that the permane...</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20hon.%20Friend%2C%20who%20I%20am%20sure%20will%20be%20able%20to%20develop%20his%20argument%20further%E2%80%94%5BHON.%20MEMBERS%3A%22Oh%22.%5D%20I%20was%20referring%20to%20the%20fact%20that%20the%20permane...</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>migrants and religion</t>
+          <t>migrants and the police</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Migrants strengthen religious communities</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>This is an unfunded mandate . To the issue itself . there was no argument from the other side that these words are pejorative . that this wo...</t>
-        </is>
+          <t>Police fail to protect migrants</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=This%20is%20an%20unfunded%20mandate%20.%20To%20the%20issue%20itself%20.%20there%20was%20no%20argument%20from%20the%20other%20side%20that%20these%20words%20are%20pejorative%20.%20that%20this%20wo...</t>
+          <t>My Lords I, too, congratulate the noble Lord, Lord McColl, on introducing this significant Bill so effectively. It reminds us that this abho...</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%20I%2C%20too%2C%20congratulate%20the%20noble%20Lord%2C%20Lord%20McColl%2C%20on%20introducing%20this%20significant%20Bill%20so%20effectively.%20It%20reminds%20us%20that%20this%20abho...</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>international students in higher education</t>
+          <t>migrants and labour market</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>International students who remain after graduation do low-skilled work</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>The hon. Gentleman has pre-empted me; I was going to deal with that at the end, but I will deal with it now. We have no plans to reintroduce...</t>
-        </is>
+          <t>Care worker visas are being abused by failing care homes</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=The%20hon.%20Gentleman%20has%20pre-empted%20me%3B%20I%20was%20going%20to%20deal%20with%20that%20at%20the%20end%2C%20but%20I%20will%20deal%20with%20it%20now.%20We%20have%20no%20plans%20to%20reintroduce...</t>
+          <t>My mother's in a care home. The system will collapse without immigrants</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=My%20mother%27s%20in%20a%20care%20home.%20The%20system%20will%20collapse%20without%20immigrants</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>transparency on migration data/policies</t>
+          <t>migration and language</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Transparency exposes information that can be weaponised against migrants</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Council blunder sees redacted immigration report made public</t>
-        </is>
+          <t>ESOL funding is too expensive for taxpayers</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Council%20blunder%20sees%20redacted%20immigration%20report%20made%20public</t>
+          <t>Refugees want to learn English but we're stopping them</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Refugees%20want%20to%20learn%20English%20but%20we%27re%20stopping%20them</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>migrants and racism/xenophobia</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Right to asylum encourages uncontrolled migration</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Patel's asylum 'overhaul' won't stop migrants coming to the UK, insists caller</t>
-        </is>
+          <t>Fear of migrants is justified</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Patel%27s%20asylum%20%27overhaul%27%20won%27t%20stop%20migrants%20coming%20to%20the%20UK%2C%20insists%20caller</t>
+          <t>My Lords, I welcome what the Minister has said today, and I very much welcome what my noble friend Lord Rosser said in his response. I think...</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20welcome%20what%20the%20Minister%20has%20said%20today%2C%20and%20I%20very%20much%20welcome%20what%20my%20noble%20friend%20Lord%20Rosser%20said%20in%20his%20response.%20I%20think...</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migrants, national law, and sovereignty</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Mass influx of migrants violates the human rights of locals</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Sonya Sceats: Charity leaders must unite to combat intimidation and protect democracy</t>
-        </is>
+          <t>National law should take precedence over international law on migration</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Sonya%20Sceats%3A%20Charity%20leaders%20must%20unite%20to%20combat%20intimidation%20and%20protect%20democracy</t>
+          <t>Rwanda flights will go ahead as planned, says Downing Street</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rwanda%20flights%20will%20go%20ahead%20as%20planned%2C%20says%20Downing%20Street</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>public opinion on migration</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Public opinion supports welcoming migrants</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Anti-Trump protesters gather around UK</t>
-        </is>
+          <t>Asylum seekers should be allowed to work while waiting for a decision</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Anti-Trump%20protesters%20gather%20around%20UK</t>
+          <t>(2) The following shall be inserted after paragraph 21(2E) of Schedule 2 to the Immigration Act 1971 (c. 77) (temporary admission or release...</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=%282%29%20The%20following%20shall%20be%20inserted%20after%20paragraph%2021%282E%29%20of%20Schedule%202%20to%20the%20Immigration%20Act%201971%20%28c.%2077%29%20%28temporary%20admission%20or%20release...</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>migrants and the court system</t>
+          <t>EU migration to and from the UK</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Legal systems must protect migrants from exploitation and/or mistreatment</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>UK: Supreme Court refuses to hear Shamima Begum's appeal against 'profoundly wrong' citizenship stripping</t>
-        </is>
+          <t>EU migration enhances labour mobility and economic growth</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=UK%3A%20Supreme%20Court%20refuses%20to%20hear%20Shamima%20Begum%27s%20appeal%20against%20%27profoundly%20wrong%27%20citizenship%20stripping</t>
+          <t>My Lords, I hope the noble Lord will not tempt me to make a much longer speech than I otherwise would. I was simply saying that the regional...</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20hope%20the%20noble%20Lord%20will%20not%20tempt%20me%20to%20make%20a%20much%20longer%20speech%20than%20I%20otherwise%20would.%20I%20was%20simply%20saying%20that%20the%20regional...</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cultural impacts of migration</t>
+          <t>migrants and schools</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Migration erodes cultural identity of the migrants themselves</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>My Lords, having taken part in the previous debate, I have been sitting on these Benches, almost without break, since 3 o'clock and so I kno...</t>
-        </is>
+          <t>British children are a minority in some schools</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20having%20taken%20part%20in%20the%20previous%20debate%2C%20I%20have%20been%20sitting%20on%20these%20Benches%2C%20almost%20without%20break%2C%20since%203%20o%27clock%20and%20so%20I%20kno...</t>
+          <t>‘Schoolboy aged 30 told pupils he was married father-of-two’</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=%E2%80%98Schoolboy%20aged%2030%20told%20pupils%20he%20was%20married%20father-of-two%E2%80%99</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>transparency on migration data/policies</t>
+          <t>migrants, welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Too much transparency compromises border operations</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>My Lords, I thank noble Lords for their input to the debate. With two speakers and just under 50 detailed questions, there is no doubt that ...</t>
-        </is>
+          <t>Migration increases welfare dependency</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20thank%20noble%20Lords%20for%20their%20input%20to%20the%20debate.%20With%20two%20speakers%20and%20just%20under%2050%20detailed%20questions%2C%20there%20is%20no%20doubt%20that%20...</t>
+          <t>There is significant concern across the country about the likelihood of welfare dependency as a result of immigration from Romania and Bulga...</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=There%20is%20significant%20concern%20across%20the%20country%20about%20the%20likelihood%20of%20welfare%20dependency%20as%20a%20result%20of%20immigration%20from%20Romania%20and%20Bulga...</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>public opinion on migration</t>
+          <t>children of migrants</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>The public does not support low skilled migration to the UK</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>How do we fight the loudmouth politics of authoritarian populism?</t>
-        </is>
+          <t>Migrants’ children deserve equal access to education</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=How%20do%20we%20fight%20the%20loudmouth%20politics%20of%20authoritarian%20populism%3F</t>
+          <t>Boris Johnson meets with Ukrainian children who fled Putin’s bloodshed for sanctuary in Britain...</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Boris%20Johnson%20meets%20with%20Ukrainian%20children%20who%20fled%20Putin%E2%80%99s%20bloodshed%20for%20sanctuary%20in%20Britain...</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Illegal and legal immigration questions do overlap</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>I understand their interest in considering them separately . But I hope the membership of the Senate will consider the question of joining t...</t>
-        </is>
+          <t>Asylum seekers should be allowed to work while waiting for a decision</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=I%20understand%20their%20interest%20in%20considering%20them%20separately%20.%20But%20I%20hope%20the%20membership%20of%20the%20Senate%20will%20consider%20the%20question%20of%20joining%20t...</t>
+          <t>My Lords, Amendment 134, which I wish to support, is simple, just and proportionate in its aims. I accept that Home Office officials must, i...</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20Amendment%20134%2C%20which%20I%20wish%20to%20support%2C%20is%20simple%2C%20just%20and%20proportionate%20in%20its%20aims.%20I%20accept%20that%20Home%20Office%20officials%20must%2C%20i...</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>migrants and healthcare system</t>
+          <t>detention and deportation of migrants</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Migrant doctors and nurses save British lives</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Immigration is personal to all of us, whether we are immigrants ourselves, the descendants of immigrants, or benefit from the skills, talent...</t>
-        </is>
+          <t>Deporting asylum seekers to Rwanda is a bad idea</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Immigration%20is%20personal%20to%20all%20of%20us%2C%20whether%20we%20are%20immigrants%20ourselves%2C%20the%20descendants%20of%20immigrants%2C%20or%20benefit%20from%20the%20skills%2C%20talent...</t>
+          <t>My Lords, a legal ruling has said that the Government’s asylum processing deal with Rwanda is legal, although with a number of qualification...</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20a%20legal%20ruling%20has%20said%20that%20the%20Government%E2%80%99s%20asylum%20processing%20deal%20with%20Rwanda%20is%20legal%2C%20although%20with%20a%20number%20of%20qualification...</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>migrants and permanent residence or citizenship</t>
+          <t>migrants in sports and athletics</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Permanent settlement helps migrants integrate</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>I have here a list of all the organisations that played their part in the Clarke Report. Perhaps I could let my hon. Friend know later.&lt;p&gt;&lt;/...</t>
-        </is>
+          <t>Foreign-born athletes lack a genuine sense of national pride for their host country</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20have%20here%20a%20list%20of%20all%20the%20organisations%20that%20played%20their%20part%20in%20the%20Clarke%20Report.%20Perhaps%20I%20could%20let%20my%20hon.%20Friend%20know%20later.%3Cp%3E%3C%2F...</t>
+          <t>Stoke City: Sammy Bangoura one reason Peter Coates branded him "a disgrace"</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Stoke%20City%3A%20Sammy%20Bangoura%20one%20reason%20Peter%20Coates%20branded%20him%20%22a%20disgrace%22</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Asylum seekers are housed in the UK but not in other countries</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Labour confirms: No more housing asylum seekers on Bibby Stockholm barge</t>
-        </is>
+          <t>Migrants increase theft and property crimes</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Labour%20confirms%3A%20No%20more%20housing%20asylum%20seekers%20on%20Bibby%20Stockholm%20barge</t>
+          <t>Married international jewellery thieves jailed after £50k spree</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Married%20international%20jewellery%20thieves%20jailed%20after%20%C2%A350k%20spree</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LGBT migrants</t>
+          <t>international cooperation on migration</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>LGBT migrants need protection from persecution</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Two per cent of those claiming asylum in this country are LGBTQI+ people fleeing countries where just being themselves can be a death senten...</t>
-        </is>
+          <t>International cooperation is necessary on asylum issues</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Two%20per%20cent%20of%20those%20claiming%20asylum%20in%20this%20country%20are%20LGBTQI%2B%20people%20fleeing%20countries%20where%20just%20being%20themselves%20can%20be%20a%20death%20senten...</t>
+          <t>I will speak briefly on this matter, because most of the arguments have already been rehearsed. I am happy to support the hon. Member for We...</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20will%20speak%20briefly%20on%20this%20matter%2C%20because%20most%20of%20the%20arguments%20have%20already%20been%20rehearsed.%20I%20am%20happy%20to%20support%20the%20hon.%20Member%20for%20We...</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>migrants and crimes</t>
+          <t>family members of migrants</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Migrants are involved in arson</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Anti-immigration protests: Police reveal block of flats was evacuated after rioters torched halal supermarket in Belfast</t>
-        </is>
+          <t>Protecting family rights is a humanitarian duty</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Anti-immigration%20protests%3A%20Police%20reveal%20block%20of%20flats%20was%20evacuated%20after%20rioters%20torched%20halal%20supermarket%20in%20Belfast</t>
+          <t>Will the Leader of the House arrange for a debate on early-day motion 17 which relates to lady Kurdish hunger strikers?&lt;p&gt;&lt;/p&gt;&lt;em&gt;[That this...</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Will%20the%20Leader%20of%20the%20House%20arrange%20for%20a%20debate%20on%20early-day%20motion%2017%20which%20relates%20to%20lady%20Kurdish%20hunger%20strikers%3F%3Cp%3E%3C%2Fp%3E%3Cem%3E%5BThat%20this...</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>migrants and healthcare system</t>
+          <t>children of migrants</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Migrants work in, and strengthen, public services</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>The NHS surcharge for migrant staff is gone. Why did it take such a fight?</t>
-        </is>
+          <t>Migrants’ children need mental health support</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=The%20NHS%20surcharge%20for%20migrant%20staff%20is%20gone.%20Why%20did%20it%20take%20such%20a%20fight%3F</t>
+          <t>It is a pleasure to serve under your chairmanship, Mr Stringer, and a pleasure, as always, to follow the hon. Member for Liverpool, West Der...</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=It%20is%20a%20pleasure%20to%20serve%20under%20your%20chairmanship%2C%20Mr%20Stringer%2C%20and%20a%20pleasure%2C%20as%20always%2C%20to%20follow%20the%20hon.%20Member%20for%20Liverpool%2C%20West%20Der...</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>geopolitical impacts of migration</t>
+          <t>detention and deportation of migrants</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Migration fosters international cooperation and soft power</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Mr. MENENDEZ. Mr. President, I am rising to ask unanimous consent to 
-consider the nomination of Leopoldo Martinez. This body should confirm...</t>
-        </is>
+          <t>Deporting asylum seekers to Rwanda is a good idea</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Mr.%20MENENDEZ.%20Mr.%20President%2C%20I%20am%20rising%20to%20ask%20unanimous%20consent%20to%20%0Aconsider%20the%20nomination%20of%20Leopoldo%20Martinez.%20This%20body%20should%20confirm...</t>
+          <t>Home Office hires hangar to practice forcibly sending asylum seekers to Rwanda</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Home%20Office%20hires%20hangar%20to%20practice%20forcibly%20sending%20asylum%20seekers%20to%20Rwanda</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and racism/xenophobia</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Migrants start businesses and create jobs</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>I am talking about the number of entrepreneurs. The framework created since 1979 has led to a sharp rise in the birth rate of new businesses...</t>
-        </is>
+          <t>Migrants are racist towards locals</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20talking%20about%20the%20number%20of%20entrepreneurs.%20The%20framework%20created%20since%201979%20has%20led%20to%20a%20sharp%20rise%20in%20the%20birth%20rate%20of%20new%20businesses...</t>
+          <t>I should not have done the hon. Member for Northampton, North (Mr. Marlow) the courtesy of prolonging the debate, and thus making it more im...</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20should%20not%20have%20done%20the%20hon.%20Member%20for%20Northampton%2C%20North%20%28Mr.%20Marlow%29%20the%20courtesy%20of%20prolonging%20the%20debate%2C%20and%20thus%20making%20it%20more%20im...</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>migrants and crimes</t>
+          <t>historical and colonial responsibility towards migrants</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Migrants import illegal drugs</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Houghton-le-Spring armed robber left shop workers terrified after raid to get money for Christmas presents</t>
-        </is>
+          <t>Historical or colonial ties between nations do not justify free movement</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Houghton-le-Spring%20armed%20robber%20left%20shop%20workers%20terrified%20after%20raid%20to%20get%20money%20for%20Christmas%20presents</t>
+          <t>My Lords, it seems to me to be a disproportionate outlay of bureaucratic effort and public money for 800 officials to be at work processing ...</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20it%20seems%20to%20me%20to%20be%20a%20disproportionate%20outlay%20of%20bureaucratic%20effort%20and%20public%20money%20for%20800%20officials%20to%20be%20at%20work%20processing%20...</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>migrants and housing</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Illegal immigration has become easier than legal immigration</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>I endorse what the Minister has said, but Migrationwatch UK states that there are 875,000 illegal immigrants in the country, and that 50,000...</t>
-        </is>
+          <t>Migrants are needed to build more homes</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20endorse%20what%20the%20Minister%20has%20said%2C%20but%20Migrationwatch%20UK%20states%20that%20there%20are%20875%2C000%20illegal%20immigrants%20in%20the%20country%2C%20and%20that%2050%2C000...</t>
+          <t>Would the Minister not agree that, if we are going to be able to build enough houses for British people as well as migrants, we will need la...</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Would%20the%20Minister%20not%20agree%20that%2C%20if%20we%20are%20going%20to%20be%20able%20to%20build%20enough%20houses%20for%20British%20people%20as%20well%20as%20migrants%2C%20we%20will%20need%20la...</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and permanent residence or citizenship</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Migrants fill essential jobs locals won't take</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Pick for Britain website down moments after nation urged to sign up</t>
-        </is>
+          <t>Granting British passports to migrants discredits the British passport system</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Pick%20for%20Britain%20website%20down%20moments%20after%20nation%20urged%20to%20sign%20up</t>
+          <t>This amendment falls into two parts, and I shall, if I may, deal with them separately. The first would provide a new definition of citizen o...</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=This%20amendment%20falls%20into%20two%20parts%2C%20and%20I%20shall%2C%20if%20I%20may%2C%20deal%20with%20them%20separately.%20The%20first%20would%20provide%20a%20new%20definition%20of%20citizen%20o...</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>international students in higher education</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Asylum seekers pose a danger to the public</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Given some of the horrors of war that asylum seekers can witness, they can become desensitised to the difference between right and wrong and...</t>
-        </is>
+          <t>International study is a backdoor for migration</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Given%20some%20of%20the%20horrors%20of%20war%20that%20asylum%20seekers%20can%20witness%2C%20they%20can%20become%20desensitised%20to%20the%20difference%20between%20right%20and%20wrong%20and...</t>
+          <t>My Lords, from these Benches we strongly support the amendment of the noble Lord, Lord Hannay, and endorse everything that the noble Lord, L...</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20from%20these%20Benches%20we%20strongly%20support%20the%20amendment%20of%20the%20noble%20Lord%2C%20Lord%20Hannay%2C%20and%20endorse%20everything%20that%20the%20noble%20Lord%2C%20L...</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migrant women’s rights</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Deporting asylum seekers to Rwanda is a good idea</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>My hon. Friend makes an incredibly important point, which proves that, when the UK makes our case in international institutions such as the ...</t>
-        </is>
+          <t>Migrant women abuse protections to avoid deportation</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20hon.%20Friend%20makes%20an%20incredibly%20important%20point%2C%20which%20proves%20that%2C%20when%20the%20UK%20makes%20our%20case%20in%20international%20institutions%20such%20as%20the%20...</t>
+          <t>My Lords, I thank the noble Baroness, Lady Hayter of Kentish Town, for this debate, and her committee for its report. I also pay tribute to ...</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20thank%20the%20noble%20Baroness%2C%20Lady%20Hayter%20of%20Kentish%20Town%2C%20for%20this%20debate%2C%20and%20her%20committee%20for%20its%20report.%20I%20also%20pay%20tribute%20to%20...</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>migrants and citizenship/PR/settlement</t>
+          <t>migrants and employment</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Current national laws allow migrants to settle permanently too easily</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>That visa expires . and there is no more job available . In fact . there are Americans looking for work . That foreign worker goes home . Wh...</t>
-        </is>
+          <t>Migrants contribute to the economy</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=That%20visa%20expires%20.%20and%20there%20is%20no%20more%20job%20available%20.%20In%20fact%20.%20there%20are%20Americans%20looking%20for%20work%20.%20That%20foreign%20worker%20goes%20home%20.%20Wh...</t>
+          <t>In the few moments which are left, I hope to make some contribution to this debate. I think many of us on this side of the House felt a litt...</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=In%20the%20few%20moments%20which%20are%20left%2C%20I%20hope%20to%20make%20some%20contribution%20to%20this%20debate.%20I%20think%20many%20of%20us%20on%20this%20side%20of%20the%20House%20felt%20a%20litt...</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>migrant women’s rights</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Illegal migration undermines the rule of law</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Harry should spare a thought for his family, says ANN WIDDECOMBE</t>
-        </is>
+          <t>Migrant women are victims of gender-based violence</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Harry%20should%20spare%20a%20thought%20for%20his%20family%2C%20says%20ANN%20WIDDECOMBE</t>
+          <t>My Lords, as we have previously set out, the purpose of the Bill is to stop the boats and end the perilous journeys being made across the ch...</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20as%20we%20have%20previously%20set%20out%2C%20the%20purpose%20of%20the%20Bill%20is%20to%20stop%20the%20boats%20and%20end%20the%20perilous%20journeys%20being%20made%20across%20the%20ch...</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>migrants and housing</t>
+          <t>accountability on migration policies</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Migrants are housed in the UK but not in other countries</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Cumberland arranging homes for Afghan families as 'bridging' scheme ends</t>
-        </is>
+          <t>Governments must be accountable for crimes committed by migrants</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Cumberland%20arranging%20homes%20for%20Afghan%20families%20as%20%27bridging%27%20scheme%20ends</t>
+          <t>Jamaica deportation flight leaves but without some detainees after Court of Appeal ruling</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Jamaica%20deportation%20flight%20leaves%20but%20without%20some%20detainees%20after%20Court%20of%20Appeal%20ruling</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>climate migration</t>
+          <t>migrants and elections</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Helping climate migrants is a moral duty</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>‘It’s my calling’: Mikaela Loach, rising star of the climate crisis campaign</t>
-        </is>
+          <t>Migrants can enrich democratic participation once naturalised</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=%E2%80%98It%E2%80%99s%20my%20calling%E2%80%99%3A%20Mikaela%20Loach%2C%20rising%20star%20of%20the%20climate%20crisis%20campaign</t>
+          <t>Labour could allow settled migrants and 16 and 17-year-olds to vote</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Labour%20could%20allow%20settled%20migrants%20and%2016%20and%2017-year-olds%20to%20vote</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>migrants and assimilation</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Migrants wish to be a separate community within the State</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>I believe that I can claim to be the first Member of this House who has ever printed an election address in Urdu. I did so in the 1955 Elect...</t>
-        </is>
+          <t>Asylum seekers entering the UK from safe countries and claiming asylum should not be allowed to stay</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20believe%20that%20I%20can%20claim%20to%20be%20the%20first%20Member%20of%20this%20House%20who%20has%20ever%20printed%20an%20election%20address%20in%20Urdu.%20I%20did%20so%20in%20the%201955%20Elect...</t>
+          <t>Asylum hotels in Surrey and what happens next</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Asylum%20hotels%20in%20Surrey%20and%20what%20happens%20next</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>migrants and permanent residence or citizenship</t>
+          <t>international cooperation on migration</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Migrants exploit permanent residence to access welfare benefits</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Not for the first time, and certainly not for the last, I stand corrected.
-It is absolutely right that almost every contributor to this t...</t>
-        </is>
+          <t>International cooperation is necessary on refugee issues</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Not%20for%20the%20first%20time%2C%20and%20certainly%20not%20for%20the%20last%2C%20I%20stand%20corrected.%0D%0A%0D%0AIt%20is%20absolutely%20right%20that%20almost%20every%20contributor%20to%20this%20t...</t>
+          <t>My Lords, I thank the noble Lord, Lord Scriven, for securing this debate. I also extend my thanks to the inspectors for their helpful report...</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20thank%20the%20noble%20Lord%2C%20Lord%20Scriven%2C%20for%20securing%20this%20debate.%20I%20also%20extend%20my%20thanks%20to%20the%20inspectors%20for%20their%20helpful%20report...</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LGBT migrants</t>
+          <t>migrants and elections</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LGBT migrants need protection from persecution</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>I spent a year in an asylum hotel. I was beaten up and lived on £9 a week</t>
-        </is>
+          <t>EU migrants should not be allowed to vote in UK elections</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=I%20spent%20a%20year%20in%20an%20asylum%20hotel.%20I%20was%20beaten%20up%20and%20lived%20on%20%C2%A39%20a%20week</t>
+          <t>Tens of thousands in Cov have no say in elections</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Tens%20of%20thousands%20in%20Cov%20have%20no%20say%20in%20elections</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>migrants and housing</t>
+          <t>demographic aspects of migration</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Mass migration has outpaced house building</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Susan Aitken: Government must help us end homelessness crisis</t>
-        </is>
+          <t>Migrants weaken the national genes by marrying locals</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Susan%20Aitken%3A%20Government%20must%20help%20us%20end%20homelessness%20crisis</t>
+          <t>Why is Vivek Ramaswamy doubling down on conspiracy theories?</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Why%20is%20Vivek%20Ramaswamy%20doubling%20down%20on%20conspiracy%20theories%3F</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migrants, welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Targeted deportations deter repeat irregular entry</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Kemi Badenoch vows to set up Trump-style Removals Force</t>
-        </is>
+          <t>Migrants who claim welfare do not deserve to stay</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Kemi%20Badenoch%20vows%20to%20set%20up%20Trump-style%20Removals%20Force</t>
+          <t>My Lords, on a careful analysis, made over a series of years, it was discovered (at least, many people believe this, though I bow to the nob...</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20on%20a%20careful%20analysis%2C%20made%20over%20a%20series%20of%20years%2C%20it%20was%20discovered%20%28at%20least%2C%20many%20people%20believe%20this%2C%20though%20I%20bow%20to%20the%20nob...</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>climate migration</t>
+          <t>public opinion on migration</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Climate migrants are economic migrants in disguise</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Here’s what we need to do to avoid total climate breakdown</t>
-        </is>
+          <t>Public opinion on migration varies depending on the nationality of the migrants</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Here%E2%80%99s%20what%20we%20need%20to%20do%20to%20avoid%20total%20climate%20breakdown</t>
+          <t>My Lords, I should like to add my congratulations to the noble Lord, Lord St. Helens, upon a powerful and skilled maiden speech. It is quite...</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20should%20like%20to%20add%20my%20congratulations%20to%20the%20noble%20Lord%2C%20Lord%20St.%20Helens%2C%20upon%20a%20powerful%20and%20skilled%20maiden%20speech.%20It%20is%20quite...</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>children of migrants</t>
+          <t>migrants, welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Age assessments are unreliable and harm genuine child refugees</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>My Lords, I understand the concern that the asylum procedures should properly protect the interests of children. Children—especially unaccom...</t>
-        </is>
+          <t>Migrants contribute to the economy, so they merit resources</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20understand%20the%20concern%20that%20the%20asylum%20procedures%20should%20properly%20protect%20the%20interests%20of%20children.%20Children%E2%80%94especially%20unaccom...</t>
+          <t>£7million dedicated funding to support Afghan refugees fleeing war to resettle</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=%C2%A37million%20dedicated%20funding%20to%20support%20Afghan%20refugees%20fleeing%20war%20to%20resettle</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>migrants and terrorism</t>
+          <t>migrants, national law, and sovereignty</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Small boat arrivals could be terrorists</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>On a point of order, Madam Deputy Speaker. I have given notice to the Speaker’s Office and the hon. Member for Ashfield (Lee Anderson) of th...</t>
-        </is>
+          <t>National laws about migration are too weak because politicians are scared of being called racist</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=On%20a%20point%20of%20order%2C%20Madam%20Deputy%20Speaker.%20I%20have%20given%20notice%20to%20the%20Speaker%E2%80%99s%20Office%20and%20the%20hon.%20Member%20for%20Ashfield%20%28Lee%20Anderson%29%20of%20th...</t>
+          <t>Gordon Brown in call to delay Brexit</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Gordon%20Brown%20in%20call%20to%20delay%20Brexit</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>geopolitical impacts of migration</t>
+          <t>social integration of migrants</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Hostile states or actors are fuelling concerns about migration to create instability</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>15,000 Russian millionaires seeking to emigrate, says UK</t>
-        </is>
+          <t>Migrants actively participate in civic life</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=15%2C000%20Russian%20millionaires%20seeking%20to%20emigrate%2C%20says%20UK</t>
+          <t>Stafford entrepreneur now offers taste of Ukraine events at home</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Stafford%20entrepreneur%20now%20offers%20taste%20of%20Ukraine%20events%20at%20home</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>international students in higher education</t>
+          <t>accountability on migration policies</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>International students enrich academic environments</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>My Lords, it is a privilege to introduce this debate on a topic of such importance to the future of the country. This is a Labour-sponsored ...</t>
-        </is>
+          <t>Accountability measures delay decisive action on migration</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20it%20is%20a%20privilege%20to%20introduce%20this%20debate%20on%20a%20topic%20of%20such%20importance%20to%20the%20future%20of%20the%20country.%20This%20is%20a%20Labour-sponsored%20...</t>
+          <t>Rule by the blob is this election’s elephant in the room, says Radomir Tylecote</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rule%20by%20the%20blob%20is%20this%20election%E2%80%99s%20elephant%20in%20the%20room%2C%20says%20Radomir%20Tylecote</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>international cooperation on migration</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>International cooperation is necessary on illegal migration issues</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>I cannot, I am afraid. I am trying to reply to all hon. Members who have spoken.&lt;p&gt;&lt;/p&gt;&lt;span id="247" class="column-number" data-column-numb...</t>
-        </is>
+          <t>The asylum system is failing both migrants and British citizens alike</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20cannot%2C%20I%20am%20afraid.%20I%20am%20trying%20to%20reply%20to%20all%20hon.%20Members%20who%20have%20spoken.%3Cp%3E%3C%2Fp%3E%3Cspan%20id%3D%22247%22%20class%3D%22column-number%22%20data-column-numb...</t>
+          <t>We need to talk about immigration</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=We%20need%20to%20talk%20about%20immigration</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>demographic aspects of migration</t>
+          <t>migrants in sports and athletics</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Migrants weaken social cohesion by changing demographics</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>I have read that reply, which means nothing. Is the Minister aware the continual migration from the North-East is having a disastrous effect...</t>
-        </is>
+          <t>Migrant sports stars inspire the next generation of diverse talent</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20have%20read%20that%20reply%2C%20which%20means%20nothing.%20Is%20the%20Minister%20aware%20the%20continual%20migration%20from%20the%20North-East%20is%20having%20a%20disastrous%20effect...</t>
+          <t>Meet Liverpool target Naby Keita, the ambitious yet humble superstar whose shoulders RB Leipzig's success is built on</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Meet%20Liverpool%20target%20Naby%20Keita%2C%20the%20ambitious%20yet%20humble%20superstar%20whose%20shoulders%20RB%20Leipzig%27s%20success%20is%20built%20on</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>migrants and human rights</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Harsh border control policies violate human rights</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>I am extremely concerned about and should welcome some enlightenment on Clause 9. However, I should declare an interest as a member of the &lt;...</t>
-        </is>
+          <t>Migrants increase violent crimes</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20extremely%20concerned%20about%20and%20should%20welcome%20some%20enlightenment%20on%20Clause%209.%20However%2C%20I%20should%20declare%20an%20interest%20as%20a%20member%20of%20the%20%3C...</t>
+          <t>Manvers offender caught by his own incriminating footage</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Manvers%20offender%20caught%20by%20his%20own%20incriminating%20footage</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>migrants and human rights</t>
+          <t>migrants and housing</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Protecting the human rights of locals should be the national priority</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>We are a little ahead of time, but I will break the habit of a lifetime and not abuse my position by taking too much of the remaining time. ...</t>
-        </is>
+          <t>Asylum seekers are placed in hotels paid for by taxpayers</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=We%20are%20a%20little%20ahead%20of%20time%2C%20but%20I%20will%20break%20the%20habit%20of%20a%20lifetime%20and%20not%20abuse%20my%20position%20by%20taking%20too%20much%20of%20the%20remaining%20time.%20...</t>
+          <t>Housing asylum seekers in Essex hotel causing ‘very serious problem’, court told</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Housing%20asylum%20seekers%20in%20Essex%20hotel%20causing%20%E2%80%98very%20serious%20problem%E2%80%99%2C%20court%20told</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>migrants and the labour market</t>
+          <t>migrants and housing</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Migration increases public sector costs</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>John Redwood: Conservative voters are looking for a bold new agenda, and nothing less is going to woo them</t>
-        </is>
+          <t>Migrants drive up rents and housing shortages</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=John%20Redwood%3A%20Conservative%20voters%20are%20looking%20for%20a%20bold%20new%20agenda%2C%20and%20nothing%20less%20is%20going%20to%20woo%20them</t>
+          <t>My Lords, I congratulate the noble Lord, Lord Parekh, on initiating this debate. Having seen the list of speakers, I look forward immensely ...</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20congratulate%20the%20noble%20Lord%2C%20Lord%20Parekh%2C%20on%20initiating%20this%20debate.%20Having%20seen%20the%20list%20of%20speakers%2C%20I%20look%20forward%20immensely%20...</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migration and the economy</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Targeted deportations deter repeat irregular entry</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Many people in my constituency are angry and frustrated at Britain’s approach to illegal migration. They see hundreds of people every week g...</t>
-        </is>
+          <t>Migrants contribute significantly to the UK economy</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Many%20people%20in%20my%20constituency%20are%20angry%20and%20frustrated%20at%20Britain%E2%80%99s%20approach%20to%20illegal%20migration.%20They%20see%20hundreds%20of%20people%20every%20week%20g...</t>
+          <t>My Lords, as my noble friend Lady Hamwee has made clear, on these Benches we support Amendments 17 and 25. I am particularly pleased to see ...</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20as%20my%20noble%20friend%20Lady%20Hamwee%20has%20made%20clear%2C%20on%20these%20Benches%20we%20support%20Amendments%2017%20and%2025.%20I%20am%20particularly%20pleased%20to%20see%20...</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>migrants and schools</t>
+          <t>migrants and human rights</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Language support for migrant students benefits all learners</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>My Lords, the temptation to give my lecture gets ever stronger, but I shall resist it. I still do not regard this as a genuine experiment, b...</t>
-        </is>
+          <t>Harsh border control policies violate human rights</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20the%20temptation%20to%20give%20my%20lecture%20gets%20ever%20stronger%2C%20but%20I%20shall%20resist%20it.%20I%20still%20do%20not%20regard%20this%20as%20a%20genuine%20experiment%2C%20b...</t>
+          <t>Thank you, Mr Speaker—it is an unexpected pleasure.
+I will be voting against the Bill today. I am proud to support the reasoned amendment...</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Thank%20you%2C%20Mr%20Speaker%E2%80%94it%20is%20an%20unexpected%20pleasure.%0D%0A%0D%0AI%20will%20be%20voting%20against%20the%20Bill%20today.%20I%20am%20proud%20to%20support%20the%20reasoned%20amendment...</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>migrants and domestic violence</t>
+          <t>international students in higher education</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Migrants are victims of domestic abuse</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Family of woman found dead in car in London accuses police of failing to protect her</t>
-        </is>
+          <t>International students create jobs and boost local economies</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Family%20of%20woman%20found%20dead%20in%20car%20in%20London%20accuses%20police%20of%20failing%20to%20protect%20her</t>
+          <t>Benefits of international students outweigh costs - report</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Benefits%20of%20international%20students%20outweigh%20costs%20-%20report</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>social integration of migrants</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Integration happens through small acts of kindness</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Walking and football group helps refugees and asylum seekers feel at home in Huddersfield</t>
-        </is>
+          <t>Migrants are involved in violent crimes</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Walking%20and%20football%20group%20helps%20refugees%20and%20asylum%20seekers%20feel%20at%20home%20in%20Huddersfield</t>
+          <t>It is a pleasure to serve under your chairmanship, Mr Gray. I commend and congratulate my hon. Friend the Member for Redditch (Rachel Maclea...</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=It%20is%20a%20pleasure%20to%20serve%20under%20your%20chairmanship%2C%20Mr%20Gray.%20I%20commend%20and%20congratulate%20my%20hon.%20Friend%20the%20Member%20for%20Redditch%20%28Rachel%20Maclea...</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and schools</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Migrants are willing to work for lower pay and conditions</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Over the past four and a half years . Republicans have voted against Democratic amendments that would have added an additional 6.600 Border ...</t>
-        </is>
+          <t>Insufficient language services hinder migrant student integration</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Over%20the%20past%20four%20and%20a%20half%20years%20.%20Republicans%20have%20voted%20against%20Democratic%20amendments%20that%20would%20have%20added%20an%20additional%206.600%20Border%20...</t>
+          <t>I will elaborate on my reasoning, but it is a matter of public record that I cited the effective abolition of the grant, in so far as it was...</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20will%20elaborate%20on%20my%20reasoning%2C%20but%20it%20is%20a%20matter%20of%20public%20record%20that%20I%20cited%20the%20effective%20abolition%20of%20the%20grant%2C%20in%20so%20far%20as%20it%20was...</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>migrants and veterans</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>The UK is not hosting sufficient asylum seekers comparatively</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Leading Northern Ireland churchmen slam politicians for ‘defending rights of rivers and trees – but not unborn children’</t>
-        </is>
+          <t>Foreign-born soldiers strengthen the British military</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Leading%20Northern%20Ireland%20churchmen%20slam%20politicians%20for%20%E2%80%98defending%20rights%20of%20rivers%20and%20trees%20%E2%80%93%20but%20not%20unborn%20children%E2%80%99</t>
+          <t>Thank you, Dr Huq. It is a pleasure to serve under your chairship, and I am grateful to speak in this very important debate. In the time ava...</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Thank%20you%2C%20Dr%20Huq.%20It%20is%20a%20pleasure%20to%20serve%20under%20your%20chairship%2C%20and%20I%20am%20grateful%20to%20speak%20in%20this%20very%20important%20debate.%20In%20the%20time%20ava...</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>cultural impacts of migration</t>
+          <t>migrants and healthcare system</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Migrants weaken social cohesion by their incompatible culture</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>My Lords, I did not put my name down to speak because I did not feel that I could help much by the words that I might say. On the other hand...</t>
-        </is>
+          <t>Migrant doctors and nurses save British lives</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20did%20not%20put%20my%20name%20down%20to%20speak%20because%20I%20did%20not%20feel%20that%20I%20could%20help%20much%20by%20the%20words%20that%20I%20might%20say.%20On%20the%20other%20hand...</t>
+          <t>I beg to move,
+That leave be given to bring in a Bill to grant indefinite leave to remain to health and social care staff; and for connec...</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20beg%20to%20move%2C%0D%0A%0D%0AThat%20leave%20be%20given%20to%20bring%20in%20a%20Bill%20to%20grant%20indefinite%20leave%20to%20remain%20to%20health%20and%20social%20care%20staff%3B%20and%20for%20connec...</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>right to asylum</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>The right to asylum is fundamental under international law</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>The economy was left in a shambles . Faced with these terrible circumstances . and with continual danger for themselves and their families ....</t>
-        </is>
+          <t>Migrants are involved in crimes</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=The%20economy%20was%20left%20in%20a%20shambles%20.%20Faced%20with%20these%20terrible%20circumstances%20.%20and%20with%20continual%20danger%20for%20themselves%20and%20their%20families%20....</t>
+          <t>I beg to move, as an amendment to the Address, at the end of the Question to add: &lt;blockquote&gt;&lt;q&gt;'But humbly regret that the Gracious Speech...</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20beg%20to%20move%2C%20as%20an%20amendment%20to%20the%20Address%2C%20at%20the%20end%20of%20the%20Question%20to%20add%3A%20%3Cblockquote%3E%3Cq%3E%27But%20humbly%20regret%20that%20the%20Gracious%20Speech...</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>family members of migrants</t>
+          <t>migrants and the court system</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Family rights claims are abused for illegal entry</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Thousands of people 'pretending to live in Ireland' to help family members live in the UK</t>
-        </is>
+          <t>Migrants should have equal access to courts and legal aid</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Thousands%20of%20people%20%27pretending%20to%20live%20in%20Ireland%27%20to%20help%20family%20members%20live%20in%20the%20UK</t>
+          <t>I am not suggesting that they are not trained in their job, but that they do not have legal training sufficient to enable them to sift a gre...</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20not%20suggesting%20that%20they%20are%20not%20trained%20in%20their%20job%2C%20but%20that%20they%20do%20not%20have%20legal%20training%20sufficient%20to%20enable%20them%20to%20sift%20a%20gre...</t>
         </is>
       </c>
     </row>
@@ -1848,369 +2040,420 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Legal pathways could reduce irregular migration</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Rwanda asylum plan is lawful, High Court rules</t>
-        </is>
+          <t>Separate migration regimes within the UK would not necessarily drive up illegal immigration</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rwanda%20asylum%20plan%20is%20lawful%2C%20High%20Court%20rules</t>
+          <t>Scotland can run its own immigration system</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Scotland%20can%20run%20its%20own%20immigration%20system</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>family members of migrants</t>
+          <t>international cooperation on migration</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Family rights claims are abused for illegal entry</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>'I married Egyptian toyboy 46 years younger than me - now I want him deported'</t>
-        </is>
+          <t>International cooperation helps share migration responsibilities</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>2</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=%27I%20married%20Egyptian%20toyboy%2046%20years%20younger%20than%20me%20-%20now%20I%20want%20him%20deported%27</t>
+          <t>Starmer vows £84m aid package to stop migration crisis ‘at source’ as summit ends</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Starmer%20vows%20%C2%A384m%20aid%20package%20to%20stop%20migration%20crisis%20%E2%80%98at%20source%E2%80%99%20as%20summit%20ends</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>migrants and racism/xenophobia</t>
+          <t>migrants and welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Opposing migration is wrongly labelled as xenophobia</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>It is very difficult to follow the excellent and wise words of the right hon. Member for Leeds Central (Hilary Benn). I add my congratulatio...</t>
-        </is>
+          <t>Migrants exploit permanent residence to access welfare benefits</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=It%20is%20very%20difficult%20to%20follow%20the%20excellent%20and%20wise%20words%20of%20the%20right%20hon.%20Member%20for%20Leeds%20Central%20%28Hilary%20Benn%29.%20I%20add%20my%20congratulatio...</t>
+          <t>I am grateful for that intervention, and I recognise the complexity of the subject we are discussing. The hon. Lady has cited evidence that ...</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20grateful%20for%20that%20intervention%2C%20and%20I%20recognise%20the%20complexity%20of%20the%20subject%20we%20are%20discussing.%20The%20hon.%20Lady%20has%20cited%20evidence%20that%20...</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>geopolitical impacts of migration</t>
+          <t>climate migration</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Migrants are the soft power of hostile countries</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Chinese firms paid £15M annually to run UK asylum hotels</t>
-        </is>
+          <t>Climate change is a major driver of migration</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Chinese%20firms%20paid%20%C2%A315M%20annually%20to%20run%20UK%20asylum%20hotels</t>
+          <t>Building a strategy for an uncertain world</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Building%20a%20strategy%20for%20an%20uncertain%20world</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>deserving vs. undeserving migrant</t>
+          <t>migrants and religion</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>All migrants deserve equal treatment and rights</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Migrants 'deserve to be treated with compassion and respect' – Downing Street</t>
-        </is>
+          <t>Muslim migrants believe non-Muslims are inferior</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>2</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Migrants%20%27deserve%20to%20be%20treated%20with%20compassion%20and%20respect%27%20%E2%80%93%20Downing%20Street</t>
+          <t>Negative media narrative fuelling anti-Muslim sentiment, new poll suggests</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Negative%20media%20narrative%20fuelling%20anti-Muslim%20sentiment%2C%20new%20poll%20suggests</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>migrants, welfare, and public finance/services</t>
+          <t>EU migration to and from the UK</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Migrants' taxes help maintain public services</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>They bring their hopes and dreams and in turn . contribute . enrich and energize America . In my home state of Minnesota . immigrants have w...</t>
-        </is>
+          <t>EU migration takes jobs from local workers</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=They%20bring%20their%20hopes%20and%20dreams%20and%20in%20turn%20.%20contribute%20.%20enrich%20and%20energize%20America%20.%20In%20my%20home%20state%20of%20Minnesota%20.%20immigrants%20have%20w...</t>
+          <t>Boris Johnson pledges 'tough' Australian-style immigration scheme</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Boris%20Johnson%20pledges%20%27tough%27%20Australian-style%20immigration%20scheme</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>migrants in sports and athletics</t>
+          <t>media coverage on migration</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Young migrant athletes are often victims of exploitation by agents and scouts</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Rangers and Wolves 'tracking' 19 y/o international star as transfer race intensifies</t>
-        </is>
+          <t>Media has a pro-immigrant bias in coverage</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Rangers%20and%20Wolves%20%27tracking%27%2019%20y%2Fo%20international%20star%20as%20transfer%20race%20intensifies</t>
+          <t>The New Arrivals project – why we are reporting on asylum seekers in the UK</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=The%20New%20Arrivals%20project%20%E2%80%93%20why%20we%20are%20reporting%20on%20asylum%20seekers%20in%20the%20UK</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>demographic aspects of migration</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Legal migration is too restrictive and fuels illegality</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Congress is begrudging disaster relief to our farmers . The Nations transportation infrastructure is underfunded . and some are proposing to...</t>
-        </is>
+          <t>Migration is needed to prevent future economic problems</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>2</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Congress%20is%20begrudging%20disaster%20relief%20to%20our%20farmers%20.%20The%20Nations%20transportation%20infrastructure%20is%20underfunded%20.%20and%20some%20are%20proposing%20to...</t>
+          <t>The true, the good and the beautiful</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=The%20true%2C%20the%20good%20and%20the%20beautiful</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>international students in higher education</t>
+          <t>cultural impacts of migration</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>International students are the brightest and best</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>University of Bradford continues relationship with Bestway Foundation</t>
-        </is>
+          <t>Migration dilutes host country’s national culture</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=University%20of%20Bradford%20continues%20relationship%20with%20Bestway%20Foundation</t>
+          <t>As London luvvies belittle knife crime, white families vote with their feet</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=As%20London%20luvvies%20belittle%20knife%20crime%2C%20white%20families%20vote%20with%20their%20feet</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>detention and deportation of migrants</t>
+          <t>migrants and national identity</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Current detention practices violate human rights</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Amendments 137A, 137B, 137C and 137D relate to removal notices. They seek an assurance, if that is possible—I do not think the Bill suggests...</t>
-        </is>
+          <t>Migrants can become genuinely British</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Amendments%20137A%2C%20137B%2C%20137C%20and%20137D%20relate%20to%20removal%20notices.%20They%20seek%20an%20assurance%2C%20if%20that%20is%20possible%E2%80%94I%20do%20not%20think%20the%20Bill%20suggests...</t>
+          <t>I am sure that I agree with the noble and learned Earl. I believe that one of the matters to which attention should be devoted is the raisin...</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20sure%20that%20I%20agree%20with%20the%20noble%20and%20learned%20Earl.%20I%20believe%20that%20one%20of%20the%20matters%20to%20which%20attention%20should%20be%20devoted%20is%20the%20raisin...</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>migrants and housing</t>
+          <t>migrants, welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Rich migrants have displaced locals by buying up all of the good housing</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>I agree entirely with my hon. Friend. I think I invented the phrase “social cleansing” and sometimes I refer to it as the lowland clearances...</t>
-        </is>
+          <t>Migration increases welfare dependency</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20agree%20entirely%20with%20my%20hon.%20Friend.%20I%20think%20I%20invented%20the%20phrase%20%E2%80%9Csocial%20cleansing%E2%80%9D%20and%20sometimes%20I%20refer%20to%20it%20as%20the%20lowland%20clearances...</t>
+          <t>My hon. and learned Friend is absolutely right. One of the problems that has emerged is that the legal changes that have been made have defi...</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20hon.%20and%20learned%20Friend%20is%20absolutely%20right.%20One%20of%20the%20problems%20that%20has%20emerged%20is%20that%20the%20legal%20changes%20that%20have%20been%20made%20have%20defi...</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>migrants and the economy</t>
+          <t>migrants and veterans</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Migrants help fill labour shortages</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Oxford declared a “local authority of sanctuary” for refugees and asylum seekers – The Oxford Student</t>
-        </is>
+          <t>Migrants who serve in the armed forces deserve citizenship</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Oxford%20declared%20a%20%E2%80%9Clocal%20authority%20of%20sanctuary%E2%80%9D%20for%20refugees%20and%20asylum%20seekers%20%E2%80%93%20The%20Oxford%20Student</t>
+          <t>We have had a good and lively debate this afternoon. My hon. Friend the Member for Eastleigh (Chris Huhne) started it off by reminding the H...</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=We%20have%20had%20a%20good%20and%20lively%20debate%20this%20afternoon.%20My%20hon.%20Friend%20the%20Member%20for%20Eastleigh%20%28Chris%20Huhne%29%20started%20it%20off%20by%20reminding%20the%20H...</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Migrant exploitation must be prevented through regulation</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>'We thought slavery had gone away': African men exploited on Irish boats</t>
-        </is>
+          <t>Migrants are involved in sex offence</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=%27We%20thought%20slavery%20had%20gone%20away%27%3A%20African%20men%20exploited%20on%20Irish%20boats</t>
+          <t>On-the-run chemical attack suspect granted asylum in UK after sex offence</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=On-the-run%20chemical%20attack%20suspect%20granted%20asylum%20in%20UK%20after%20sex%20offence</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>climate migration</t>
+          <t>migrants and the police</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Climate change is a major driver of migration</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>We passed this bill 20 to 1 in the Agriculture Committee . I told the majority leader the other day . when he came for our markup in the com...</t>
-        </is>
+          <t>Police with migrant backgrounds protect criminal migrants</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>2</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=We%20passed%20this%20bill%2020%20to%201%20in%20the%20Agriculture%20Committee%20.%20I%20told%20the%20majority%20leader%20the%20other%20day%20.%20when%20he%20came%20for%20our%20markup%20in%20the%20com...</t>
+          <t>Police officer who falsified documents to aid visa bid 'would have been sacked'</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Police%20officer%20who%20falsified%20documents%20to%20aid%20visa%20bid%20%27would%20have%20been%20sacked%27</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>international students</t>
+          <t>historical and colonial responsibility towards migrants</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>International students compete with locals for housing</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>He was to have left the US for final interviews and processing but is now uncertain . He has an appointment in UC Davis Plant Sciences Depar...</t>
-        </is>
+          <t>Countries should welcome migrants due to past exploitation</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=He%20was%20to%20have%20left%20the%20US%20for%20final%20interviews%20and%20processing%20but%20is%20now%20uncertain%20.%20He%20has%20an%20appointment%20in%20UC%20Davis%20Plant%20Sciences%20Depar...</t>
+          <t>Is the hon. Gentleman aware that this is the first time the right hon. Gentleman has specifically denied the share of responsibility of this...</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Is%20the%20hon.%20Gentleman%20aware%20that%20this%20is%20the%20first%20time%20the%20right%20hon.%20Gentleman%20has%20specifically%20denied%20the%20share%20of%20responsibility%20of%20this...</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>migrants and national identity</t>
+          <t>migrants, economy, and labour market</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Migration dilutes national heritage</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Andrew Pakes MP: ‘We need blue-collar Labour, not Blue Labour’ – LabourList</t>
-        </is>
+          <t>Migrants are willing to work for lower pay and conditions</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Andrew%20Pakes%20MP%3A%20%E2%80%98We%20need%20blue-collar%20Labour%2C%20not%20Blue%20Labour%E2%80%99%20%E2%80%93%20LabourList</t>
+          <t>I certainly note that point, and I quite understand where it comes from, given the constituency my hon. Friend represents. I will ensure tha...</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20certainly%20note%20that%20point%2C%20and%20I%20quite%20understand%20where%20it%20comes%20from%2C%20given%20the%20constituency%20my%20hon.%20Friend%20represents.%20I%20will%20ensure%20tha...</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>demographic aspects of migration</t>
+          <t>international students in higher education</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>The country is full</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>As the Home Secretary said, quite a number of these people were born there. We cannot go back into history. We cannot let in all who had any...</t>
-        </is>
+          <t>International study is a backdoor for migration</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=As%20the%20Home%20Secretary%20said%2C%20quite%20a%20number%20of%20these%20people%20were%20born%20there.%20We%20cannot%20go%20back%20into%20history.%20We%20cannot%20let%20in%20all%20who%20had%20any...</t>
+          <t>Migration likely to be a problem for ‘years to come’, says minister</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Migration%20likely%20to%20be%20a%20problem%20for%20%E2%80%98years%20to%20come%E2%80%99%2C%20says%20minister</t>
         </is>
       </c>
     </row>
@@ -2222,435 +2465,495 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Too much transparency compromises border operations</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>John Healey was told blackout on Afghans was probably unjustified</t>
-        </is>
+          <t>Transparency provides information that protects society from the harm caused by migrants</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>2</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=John%20Healey%20was%20told%20blackout%20on%20Afghans%20was%20probably%20unjustified</t>
+          <t>I hope I made it clear that I was referring to assisted passages. The assisted passage scheme to Australia plays a very big part and enables...</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20hope%20I%20made%20it%20clear%20that%20I%20was%20referring%20to%20assisted%20passages.%20The%20assisted%20passage%20scheme%20to%20Australia%20plays%20a%20very%20big%20part%20and%20enables...</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>historical and colonial responsibility towards migrants</t>
+          <t>migrants and crimes</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Colonial obligation is outdated and irrelevant today</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>The island community feeling 'lost' in Sussex</t>
-        </is>
+          <t>Migrants are involved in money laundering</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>2</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=The%20island%20community%20feeling%20%27lost%27%20in%20Sussex</t>
+          <t>Fraudster who found properties for drug and prostitution gangs is jailed</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Fraudster%20who%20found%20properties%20for%20drug%20and%20prostitution%20gangs%20is%20jailed</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>social integration of migrants</t>
+          <t>demographic aspects of migration</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Migrants actively participate in civic life</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>How a charity is helping people from Hong Kong adjust to life in Southampton</t>
-        </is>
+          <t>Migrants weaken the national identity by changing demographics</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>2</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=How%20a%20charity%20is%20helping%20people%20from%20Hong%20Kong%20adjust%20to%20life%20in%20Southampton</t>
+          <t>I believe that the right hon. and learned Gentleman is in error. As I understand the position, this is the gross annual addition including—a...</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20believe%20that%20the%20right%20hon.%20and%20learned%20Gentleman%20is%20in%20error.%20As%20I%20understand%20the%20position%2C%20this%20is%20the%20gross%20annual%20addition%20including%E2%80%94a...</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>migrants and housing</t>
+          <t>asylum seeking</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Migrants drive up rents and housing shortages</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Accommodation pressures as 300 more Ukraine refugees expected in Lincolnshire</t>
-        </is>
+          <t>Asylum seekers entering the UK from safe countries and claiming asylum should not be allowed to stay</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>2</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Accommodation%20pressures%20as%20300%20more%20Ukraine%20refugees%20expected%20in%20Lincolnshire</t>
+          <t>Government plans to tackle asylum seeker backlog labelled 'propaganda' and a 'distraction'</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Government%20plans%20to%20tackle%20asylum%20seeker%20backlog%20labelled%20%27propaganda%27%20and%20a%20%27distraction%27</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>effectiveness of migration policy</t>
+          <t>migrants, economy, and labour market</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Effective migration policy supports economic growth</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>It would provide paychecks and backpay to Federal workers . It would provide needed disaster recovery funding . It would deliver all seven o...</t>
-        </is>
+          <t>Migrants fill essential jobs locals won’t take</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=It%20would%20provide%20paychecks%20and%20backpay%20to%20Federal%20workers%20.%20It%20would%20provide%20needed%20disaster%20recovery%20funding%20.%20It%20would%20deliver%20all%20seven%20o...</t>
+          <t>Refugees could work in rubbish collection to fill Surrey HGV driver shortage</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Refugees%20could%20work%20in%20rubbish%20collection%20to%20fill%20Surrey%20HGV%20driver%20shortage</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>migrants and economy, and labour market</t>
+          <t>migrants, welfare, and public finance/services</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Tying a worker’s visa to a single employer enables exploitation</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>It is a pleasure to serve under your chairmanship, Mr Hosie, and to see the two rapid-risers of 2015 and 2017 on the Front Benches. I want t...</t>
-        </is>
+          <t>Migrants are denied access to social welfare</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>2</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=It%20is%20a%20pleasure%20to%20serve%20under%20your%20chairmanship%2C%20Mr%20Hosie%2C%20and%20to%20see%20the%20two%20rapid-risers%20of%202015%20and%202017%20on%20the%20Front%20Benches.%20I%20want%20t...</t>
+          <t>&lt;strong&gt;Q&lt;/strong&gt;&lt;strong&gt;&lt;QNum HRSContentId="{95BD4BBF-67E7-4119-A7DC-4DB1D9E90648}"&gt; &lt;/QNum&gt;&lt;/strong&gt; And so are your children, so your ch...</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=%3Cstrong%3EQ%3C%2Fstrong%3E%3Cstrong%3E%3CQNum%20HRSContentId%3D%22%7B95BD4BBF-67E7-4119-A7DC-4DB1D9E90648%7D%22%3E%20%3C%2FQNum%3E%3C%2Fstrong%3E%20And%20so%20are%20your%20children%2C%20so%20your%20ch...</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>cultural impacts of migration</t>
+          <t>international students in higher education</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Migrants embrace local customs through integration</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Ukrainian refugees in Dorset celebrate their first Christmas in England</t>
-        </is>
+          <t>International students contribute to brain drain from home countries</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>2</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Ukrainian%20refugees%20in%20Dorset%20celebrate%20their%20first%20Christmas%20in%20England</t>
+          <t>Sunak risks Cabinet battle over plans to crack down on foreign student numbers</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Sunak%20risks%20Cabinet%20battle%20over%20plans%20to%20crack%20down%20on%20foreign%20student%20numbers</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>migrants, economy, and labour market</t>
+          <t>migrants and police</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Migrants are willing to work for lower pay and conditions</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Hispanics or whites who are citizens of this country . Perhaps . Mr. President . that is what galls me the most about this tortuously slow p...</t>
-        </is>
+          <t>Police with migrant backgrounds protect criminal migrants</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>2</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Hispanics%20or%20whites%20who%20are%20citizens%20of%20this%20country%20.%20Perhaps%20.%20Mr.%20President%20.%20that%20is%20what%20galls%20me%20the%20most%20about%20this%20tortuously%20slow%20p...</t>
+          <t>Matters are getting worse. I do not accept the arguments. In answer to the question on consultation I can say that I am not aware there was ...</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Matters%20are%20getting%20worse.%20I%20do%20not%20accept%20the%20arguments.%20In%20answer%20to%20the%20question%20on%20consultation%20I%20can%20say%20that%20I%20am%20not%20aware%20there%20was%20...</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>EU migration to and from the UK</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>It is easier to control the much higher number of legal migrants</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>As mass migration has been shown to depress GDP per capita, and as it is clear that it is easier to control the much higher number of legal ...</t>
-        </is>
+          <t>EU migration takes jobs from local workers</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>2</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=As%20mass%20migration%20has%20been%20shown%20to%20depress%20GDP%20per%20capita%2C%20and%20as%20it%20is%20clear%20that%20it%20is%20easier%20to%20control%20the%20much%20higher%20number%20of%20legal%20...</t>
+          <t>Boris Johnson pledges Australian-style points based immigration system</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Boris%20Johnson%20pledges%20Australian-style%20points%20based%20immigration%20system</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>transparency on migration policies</t>
+          <t>geopolitical impacts of migration</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Transparency builds trust in migration policy</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>To ensure that the numbers DHS gives us are sound . this bill . Mr. Speaker . requires that the Department give the Government Accountabilit...</t>
-        </is>
+          <t>Migrants are used as pawns in geopolitical conflicts</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>2</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=To%20ensure%20that%20the%20numbers%20DHS%20gives%20us%20are%20sound%20.%20this%20bill%20.%20Mr.%20Speaker%20.%20requires%20that%20the%20Department%20give%20the%20Government%20Accountabilit...</t>
+          <t>Putin 'pushing migrants to Britain' in an attempt to overwhelm borders</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Putin%20%27pushing%20migrants%20to%20Britain%27%20in%20an%20attempt%20to%20overwhelm%20borders</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>media coverage on migration</t>
+          <t>children of migrants</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Mainstream media censors negative news about migrants</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>The far right has turned on the press for a reason</t>
-        </is>
+          <t>Children of migrants deserve equal access to education</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>2</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=The%20far%20right%20has%20turned%20on%20the%20press%20for%20a%20reason</t>
+          <t>Appropriate support is provided to asylum seekers who would otherwise be destitute while applications are outstanding. Asylum seekers have a...</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=Appropriate%20support%20is%20provided%20to%20asylum%20seekers%20who%20would%20otherwise%20be%20destitute%20while%20applications%20are%20outstanding.%20Asylum%20seekers%20have%20a...</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>migrants in sports and athletics</t>
+          <t>migrants and permanent residence or citizenship</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>International sports migration reflects the globalised nature of modern athletics</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>Cricket: St Annes Cricket Club building strongly, Croft on Roses century</t>
-        </is>
+          <t>Current national laws allow migrants to settle permanently too easily</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Cricket%3A%20St%20Annes%20Cricket%20Club%20building%20strongly%2C%20Croft%20on%20Roses%20century</t>
+          <t>Portuguese immigration to UK at 13 year low</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Portuguese%20immigration%20to%20UK%20at%2013%20year%20low</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>migrants and human rights</t>
+          <t>detention and deportation of migrants</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Human rights claims by migrants are often exaggerated</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>I am most grateful for the opportunity to respond to the motion. The Human Rights Act is a statute that rarely receives a good word and is s...</t>
-        </is>
+          <t>Voluntary return programmes are more humane than forced deportation</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20am%20most%20grateful%20for%20the%20opportunity%20to%20respond%20to%20the%20motion.%20The%20Human%20Rights%20Act%20is%20a%20statute%20that%20rarely%20receives%20a%20good%20word%20and%20is%20s...</t>
+          <t>Derwentside detention centre: Protest held for International Women's Day</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Derwentside%20detention%20centre%3A%20Protest%20held%20for%20International%20Women%27s%20Day</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>small boats and Channel crossings</t>
+          <t>accountability on migration policies</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Increased law enforcement action and disruption is already showing some indication of pressure on the business model of the gangs</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>As the right hon. Member is aware, the Home Office discharges its statutory duty to provide accommodation and to support destitute asylum se...</t>
-        </is>
+          <t>Governments must be accountable for the demographic impacts of migration</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>2</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=As%20the%20right%20hon.%20Member%20is%20aware%2C%20the%20Home%20Office%20discharges%20its%20statutory%20duty%20to%20provide%20accommodation%20and%20to%20support%20destitute%20asylum%20se...</t>
+          <t>My Lords, I first thank the Government Whips for facilitating my substitution for my noble friend Lady Ludford, who is regrettably ill today...</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20first%20thank%20the%20Government%20Whips%20for%20facilitating%20my%20substitution%20for%20my%20noble%20friend%20Lady%20Ludford%2C%20who%20is%20regrettably%20ill%20today...</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>legal vs. illegal immigration</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Asylum seekers should not be allowed to work while waiting for a decision</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr">
-        <is>
-          <t>Don’t come to England – there’s nothing here, warns Channel migrant</t>
-        </is>
+          <t>Illegal migrants take advantage of weak enforcement</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Don%E2%80%99t%20come%20to%20England%20%E2%80%93%20there%E2%80%99s%20nothing%20here%2C%20warns%20Channel%20migrant</t>
+          <t>I thank noble Baroness, Lady Lister, for putting forward Amendments 68 and 70, to which I have added my name. I also support Amendment 76A t...</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=I%20thank%20noble%20Baroness%2C%20Lady%20Lister%2C%20for%20putting%20forward%20Amendments%2068%20and%2070%2C%20to%20which%20I%20have%20added%20my%20name.%20I%20also%20support%20Amendment%2076A%20t...</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>international students in higher education</t>
+          <t>detention and deportation of migrants</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>International students are valued and valuable</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr">
-        <is>
-          <t>My Lords, I have added my name to the amendment, as I did in Committee. I add my regrets that the noble Lord, Lord Patten, is not here and w...</t>
-        </is>
+          <t>Detention fails to stop illegal immigration</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>2</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20have%20added%20my%20name%20to%20the%20amendment%2C%20as%20I%20did%20in%20Committee.%20I%20add%20my%20regrets%20that%20the%20noble%20Lord%2C%20Lord%20Patten%2C%20is%20not%20here%20and%20w...</t>
+          <t>Asylum seeker escapes Dungavel detention centre clinging on to underside of van</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Asylum%20seeker%20escapes%20Dungavel%20detention%20centre%20clinging%20on%20to%20underside%20of%20van</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>cultural impacts of migration</t>
+          <t>migration and language</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Integration programs foster harmony between migrants and locals</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>It is often difficult for one who has newly come to our shores to handle the conflict between attachment to the old country and fealty to th...</t>
-        </is>
+          <t>Migrants who do not speak English isolate themselves in enclaves</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>2</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=It%20is%20often%20difficult%20for%20one%20who%20has%20newly%20come%20to%20our%20shores%20to%20handle%20the%20conflict%20between%20attachment%20to%20the%20old%20country%20and%20fealty%20to%20th...</t>
+          <t>My hon. Friend makes the important point that we recognised the importance of Syrian refugees being able to speak English, but we have not d...</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20hon.%20Friend%20makes%20the%20important%20point%20that%20we%20recognised%20the%20importance%20of%20Syrian%20refugees%20being%20able%20to%20speak%20English%2C%20but%20we%20have%20not%20d...</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>legal vs. illegal immigration</t>
+          <t>migrants and national identity</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Illegal immigrants take advantage of weak enforcement</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr">
-        <is>
-          <t>Otherwise . I am afraid the Congress and the administration will have an excuse to put this issue aside and it will be years again . literal...</t>
-        </is>
+          <t>Migrants erode traditional national customs</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>2</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=us_congress_speech&amp;title=Otherwise%20.%20I%20am%20afraid%20the%20Congress%20and%20the%20administration%20will%20have%20an%20excuse%20to%20put%20this%20issue%20aside%20and%20it%20will%20be%20years%20again%20.%20literal...</t>
+          <t>Yes, I love my Cornwall holidays — but what’s the damage?</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Yes%2C%20I%20love%20my%20Cornwall%20holidays%20%E2%80%94%20but%20what%E2%80%99s%20the%20damage%3F</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>asylum seeking</t>
+          <t>migrants and human rights</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Asylum seekers are not criminals</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr">
-        <is>
-          <t>My Lords, I am a former chairman of the Refugee Council. Like many noble Lords, I am deeply perturbed by the situation which some people—my ...</t>
-        </is>
+          <t>Protecting the human rights of locals should be the national priority</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>2</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=My%20Lords%2C%20I%20am%20a%20former%20chairman%20of%20the%20Refugee%20Council.%20Like%20many%20noble%20Lords%2C%20I%20am%20deeply%20perturbed%20by%20the%20situation%20which%20some%20people%E2%80%94my%20...</t>
+          <t>Knife-wielding terrorists have targeted Brits four times in eight months - this must stop</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=Knife-wielding%20terrorists%20have%20targeted%20Brits%20four%20times%20in%20eight%20months%20-%20this%20must%20stop</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>migrants, welfare, and public finance/services</t>
+          <t>historical and colonial responsibility towards migrants</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Migration causes longer waits for public services</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>LETTER TO THE EDITOR: Black Friday and tax cuts</t>
-        </is>
+          <t>Immigration controls on citizens of former colonies are racist policies</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>2</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=articles&amp;title=LETTER%20TO%20THE%20EDITOR%3A%20Black%20Friday%20and%20tax%20cuts</t>
+          <t>The procedure which you have outlined, Sir Gordon, is certainly convenient to hon. Members on this side of the Committee and I am sure that ...</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>https://mignar.streamlit.app/Narratives_on_Articles?source_table=uk_parliament_contributions&amp;title=The%20procedure%20which%20you%20have%20outlined%2C%20Sir%20Gordon%2C%20is%20certainly%20convenient%20to%20hon.%20Members%20on%20this%20side%20of%20the%20Committee%20and%20I%20am%20sure%20that%20...</t>
         </is>
       </c>
     </row>

</xml_diff>